<commit_message>
reorganisation fiche dans groupe et theme et famille
</commit_message>
<xml_diff>
--- a/fiches indicateurs.xlsx
+++ b/fiches indicateurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="indicateurs" sheetId="1" state="visible" r:id="rId3"/>
@@ -1871,6 +1871,18 @@
     <t xml:space="preserve">aide à la décision</t>
   </si>
   <si>
+    <t xml:space="preserve">Robustesse et résilience technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Évaluer la capacité de production en période sèche et la présence de dispositifs de secours (stockage, interconnexion) pour garantir la continuité du service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagnostic &amp; Modulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guide la mise en conformité légale et les actions de protection réglementaire.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Poids stratégique de la desserte</t>
   </si>
   <si>
@@ -1878,18 +1890,6 @@
   </si>
   <si>
     <t xml:space="preserve">Définit les priorités d'investissement et l'importance socio-économique de la ressource.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Robustesse et résilience technique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Évaluer la capacité de production en période sèche et la présence de dispositifs de secours (stockage, interconnexion) pour garantir la continuité du service.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diagnostic &amp; Modulation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guide la mise en conformité légale et les actions de protection réglementaire.</t>
   </si>
   <si>
     <t xml:space="preserve">Sécurisation sanitaire et réglementaire</t>
@@ -8713,11 +8713,11 @@
         <v>608</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="1" t="s">
         <v>609</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -8726,28 +8726,28 @@
       <c r="D2" s="1" t="s">
         <v>610</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>495</v>
+      <c r="E2" s="12" t="s">
+        <v>611</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>612</v>
+      <c r="B3" s="12" t="s">
+        <v>613</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>613</v>
-      </c>
-      <c r="E3" s="12" t="s">
         <v>614</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>495</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>615</v>
@@ -8787,7 +8787,7 @@
         <v>620</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>621</v>
@@ -8847,7 +8847,7 @@
         <v>630</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>631</v>
@@ -9013,7 +9013,7 @@
         <v>656</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>657</v>
@@ -9300,10 +9300,10 @@
         <v>26</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="F2" s="1"/>
       <c r="H2" s="1"/>
@@ -9316,10 +9316,10 @@
         <v>44</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="F3" s="1"/>
       <c r="H3" s="1"/>
@@ -9332,10 +9332,10 @@
         <v>53</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" s="1"/>
@@ -9364,10 +9364,10 @@
         <v>71</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="1"/>
@@ -9380,10 +9380,10 @@
         <v>80</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="1"/>

</xml_diff>

<commit_message>
fix : mise à jour de la donnees BDSSNC tous les mois
</commit_message>
<xml_diff>
--- a/fiches indicateurs.xlsx
+++ b/fiches indicateurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="indicateurs" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1862" uniqueCount="702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1862" uniqueCount="703">
   <si>
     <t xml:space="preserve">fiche_indicateur</t>
   </si>
@@ -1408,6 +1408,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://georep.nc/node/1323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tous les mois</t>
   </si>
   <si>
     <t xml:space="preserve">Informations brutes géologiques et techniques des ouvrages souterrains – DIMENC/SGNC</t>
@@ -6526,16 +6529,16 @@
         <v>304</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>305</v>
+        <v>459</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>305</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6543,13 +6546,13 @@
         <v>128</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>428</v>
@@ -6561,16 +6564,16 @@
         <v>304</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -6607,45 +6610,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>118</v>
@@ -6655,448 +6658,448 @@
     </row>
     <row r="3" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>118</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>20</v>
@@ -7105,62 +7108,62 @@
         <v>20</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>118</v>
@@ -7169,19 +7172,19 @@
     </row>
     <row r="24" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>541</v>
-      </c>
       <c r="E24" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>118</v>
@@ -7190,290 +7193,290 @@
     </row>
     <row r="25" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>287</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>288</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>118</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>118</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>289</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>290</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>291</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>292</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>294</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>295</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>298</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7520,7 +7523,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -7538,7 +7541,7 @@
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7869,7 +7872,7 @@
         <v>104</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>106</v>
@@ -7901,7 +7904,7 @@
         <v>33</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7924,7 +7927,7 @@
         <v>33</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7967,7 +7970,7 @@
         <v>33</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8030,7 +8033,7 @@
         <v>33</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8287,7 +8290,7 @@
         <v>128</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>33</v>
@@ -8413,7 +8416,7 @@
         <v>34</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8530,7 +8533,7 @@
         <v>7</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>33</v>
@@ -8563,25 +8566,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8595,16 +8598,16 @@
         <v>25</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="I2" s="1"/>
     </row>
@@ -8619,16 +8622,16 @@
         <v>25</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="I3" s="1"/>
     </row>
@@ -8643,16 +8646,16 @@
         <v>160</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="I4" s="1"/>
     </row>
@@ -8667,13 +8670,13 @@
         <v>160</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="I5" s="1"/>
     </row>
@@ -8688,13 +8691,13 @@
         <v>224</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="I6" s="1"/>
     </row>
@@ -8706,19 +8709,19 @@
         <v>246</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>160</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I7" s="1"/>
     </row>
@@ -8733,13 +8736,13 @@
         <v>160</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -8773,25 +8776,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8799,19 +8802,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8819,19 +8822,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8839,19 +8842,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8859,19 +8862,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8879,19 +8882,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8899,19 +8902,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8919,19 +8922,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8939,19 +8942,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8959,19 +8962,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8979,19 +8982,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8999,19 +9002,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9019,19 +9022,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9039,22 +9042,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9062,22 +9065,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9085,19 +9088,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9105,19 +9108,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>279</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
     </row>
   </sheetData>
@@ -9146,145 +9149,145 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>203</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9364,10 +9367,10 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="5"/>
@@ -9384,7 +9387,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="F2" s="1"/>
       <c r="H2" s="1"/>
@@ -9400,7 +9403,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F3" s="1"/>
       <c r="H3" s="1"/>
@@ -9416,7 +9419,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" s="1"/>
@@ -9432,7 +9435,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>
@@ -9448,7 +9451,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="1"/>
@@ -9464,7 +9467,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="1"/>
@@ -9480,7 +9483,7 @@
         <v>3</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1"/>
@@ -9496,7 +9499,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F9" s="1"/>
       <c r="H9" s="1"/>
@@ -9512,7 +9515,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1"/>
@@ -9528,7 +9531,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1"/>
@@ -9544,7 +9547,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="5"/>
@@ -9561,7 +9564,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="5"/>
@@ -9578,7 +9581,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="5"/>
@@ -9595,7 +9598,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F15" s="1"/>
       <c r="H15" s="1"/>
@@ -9605,13 +9608,13 @@
         <v>104</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1"/>
@@ -9627,7 +9630,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1"/>
@@ -9643,7 +9646,7 @@
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F18" s="1"/>
       <c r="H18" s="1"/>
@@ -9659,7 +9662,7 @@
         <v>9</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9673,7 +9676,7 @@
         <v>8</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -9689,7 +9692,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9703,7 +9706,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9717,7 +9720,7 @@
         <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9731,7 +9734,7 @@
         <v>8</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9745,7 +9748,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9759,7 +9762,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9773,7 +9776,7 @@
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9787,7 +9790,7 @@
         <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9801,7 +9804,7 @@
         <v>12</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9815,7 +9818,7 @@
         <v>12</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9829,7 +9832,7 @@
         <v>15</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9843,7 +9846,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9857,7 +9860,7 @@
         <v>13</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9871,7 +9874,7 @@
         <v>14</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9885,7 +9888,7 @@
         <v>14</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9899,7 +9902,7 @@
         <v>13</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9913,7 +9916,7 @@
         <v>13</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9927,7 +9930,7 @@
         <v>16</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update : ajout des information sur la donnée BBR disponible sur le GEOREP depuis le 12 juin 2026
</commit_message>
<xml_diff>
--- a/fiches indicateurs.xlsx
+++ b/fiches indicateurs.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1862" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="706">
   <si>
     <t xml:space="preserve">fiche_indicateur</t>
   </si>
@@ -1022,10 +1022,43 @@
     <t xml:space="preserve">Les typologies de captages doivent être standardisées pour assurer une comparaison cohérente ; certaines informations sont descriptives et susceptibles d'évoluer sans impact direct sur la criticité. Verifier que la données est bien à jour du GEOREP.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bilan Besoin Ressource (nom à vérifier)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bilan DAVAR diffusion interne – contacter DAVAR</t>
+    <t xml:space="preserve">Bilan Besoin Ressource</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.arcgis.com/home/item.html?id=6d48f295daf5471a842054d9e050765d</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">La couche BBR (bilan besoin / ressources) est calculée à partir des débits caractéristiques d’étiage médian (DCE2) auquel sont soustraits l'ensemble des </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">prélèvements d’eau autorisés</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://georep.nc/actualites/nouvelle-donnee-en-hydrologie-le-bilan-besoin-ressource</t>
   </si>
   <si>
     <t xml:space="preserve">Donnée issue d’un modèle nécessitant validation et mise à jour régulière.</t>
@@ -1816,6 +1849,9 @@
     <t xml:space="preserve">si utilisation du 200 000</t>
   </si>
   <si>
+    <t xml:space="preserve">Bilan Besoin Ressource (nom à vérifier)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Base de données ATYA (nom à vérifier)</t>
   </si>
   <si>
@@ -2189,7 +2225,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2215,6 +2251,13 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -2280,7 +2323,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2301,15 +2344,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2325,11 +2372,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5471,7 +5518,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
@@ -5485,10 +5532,13 @@
         <v>301</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>317</v>
+        <v>331</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>312</v>
+        <v>303</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>304</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>305</v>
@@ -5496,11 +5546,14 @@
       <c r="I7" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>331</v>
+      <c r="J7" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>333</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5508,7 +5561,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>300</v>
@@ -5526,10 +5579,10 @@
         <v>305</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5537,16 +5590,16 @@
         <v>100</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>303</v>
@@ -5555,13 +5608,13 @@
         <v>304</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>306</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5569,13 +5622,13 @@
         <v>101</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>317</v>
@@ -5584,7 +5637,7 @@
         <v>303</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>305</v>
@@ -5593,10 +5646,10 @@
         <v>306</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5604,13 +5657,13 @@
         <v>102</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>317</v>
@@ -5619,7 +5672,7 @@
         <v>303</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>305</v>
@@ -5628,10 +5681,10 @@
         <v>306</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5639,13 +5692,13 @@
         <v>103</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>317</v>
@@ -5654,7 +5707,7 @@
         <v>318</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>305</v>
@@ -5663,10 +5716,10 @@
         <v>306</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5674,16 +5727,16 @@
         <v>104</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>303</v>
@@ -5692,16 +5745,16 @@
         <v>304</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5709,13 +5762,13 @@
         <v>105</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>317</v>
@@ -5733,10 +5786,10 @@
         <v>306</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5744,16 +5797,16 @@
         <v>106</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>303</v>
@@ -5768,7 +5821,7 @@
         <v>306</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5776,16 +5829,16 @@
         <v>107</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>303</v>
@@ -5794,16 +5847,16 @@
         <v>304</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5811,16 +5864,16 @@
         <v>108</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>303</v>
@@ -5829,16 +5882,16 @@
         <v>304</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5846,16 +5899,16 @@
         <v>109</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>303</v>
@@ -5864,16 +5917,16 @@
         <v>304</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5881,16 +5934,16 @@
         <v>110</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>303</v>
@@ -5899,16 +5952,16 @@
         <v>304</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5916,34 +5969,34 @@
         <v>111</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>303</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5951,34 +6004,34 @@
         <v>112</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>303</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>305</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5986,13 +6039,13 @@
         <v>113</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>311</v>
@@ -6010,10 +6063,10 @@
         <v>306</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6021,16 +6074,16 @@
         <v>114</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>303</v>
@@ -6045,10 +6098,10 @@
         <v>306</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6056,37 +6109,37 @@
         <v>115</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>303</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>410</v>
+        <v>345</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>412</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6094,13 +6147,13 @@
         <v>116</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>317</v>
@@ -6109,7 +6162,7 @@
         <v>318</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>305</v>
@@ -6118,10 +6171,10 @@
         <v>306</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6129,13 +6182,13 @@
         <v>117</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>317</v>
@@ -6144,7 +6197,7 @@
         <v>318</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>305</v>
@@ -6153,10 +6206,10 @@
         <v>306</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6164,16 +6217,16 @@
         <v>118</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>303</v>
@@ -6188,10 +6241,10 @@
         <v>306</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6199,16 +6252,16 @@
         <v>119</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>303</v>
@@ -6223,10 +6276,10 @@
         <v>306</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6234,16 +6287,16 @@
         <v>120</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>303</v>
@@ -6258,10 +6311,10 @@
         <v>306</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6269,16 +6322,16 @@
         <v>129</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>303</v>
@@ -6287,16 +6340,16 @@
         <v>304</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6304,16 +6357,16 @@
         <v>121</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>303</v>
@@ -6328,10 +6381,10 @@
         <v>306</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6339,7 +6392,7 @@
         <v>122</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>300</v>
@@ -6357,10 +6410,10 @@
         <v>306</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="29.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6368,16 +6421,16 @@
         <v>123</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="E33" s="6" t="s">
-        <v>440</v>
+      <c r="E33" s="7" t="s">
+        <v>442</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>303</v>
@@ -6392,13 +6445,13 @@
         <v>306</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6406,16 +6459,16 @@
         <v>124</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>303</v>
@@ -6427,13 +6480,13 @@
         <v>305</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6441,16 +6494,16 @@
         <v>125</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>303</v>
@@ -6462,13 +6515,13 @@
         <v>305</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6476,16 +6529,16 @@
         <v>126</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>301</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>303</v>
@@ -6500,10 +6553,10 @@
         <v>306</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6511,7 +6564,7 @@
         <v>127</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>300</v>
@@ -6520,7 +6573,7 @@
         <v>301</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>303</v>
@@ -6529,16 +6582,16 @@
         <v>304</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>305</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6546,16 +6599,16 @@
         <v>128</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>303</v>
@@ -6564,22 +6617,23 @@
         <v>304</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>306</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L38"/>
   <hyperlinks>
-    <hyperlink ref="E33" r:id="rId1" display="https://georep-dtsi-sgt.opendata.arcgis.com/documents/d7ab36bb69954aea882a63993428357a/about"/>
+    <hyperlink ref="J7" r:id="rId1" display="prélèvements d’eau autorisés"/>
+    <hyperlink ref="E33" r:id="rId2" display="https://georep-dtsi-sgt.opendata.arcgis.com/documents/d7ab36bb69954aea882a63993428357a/about"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -6588,7 +6642,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -6610,496 +6664,496 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>469</v>
+        <v>470</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>471</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>475</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>476</v>
+      <c r="C2" s="9" t="s">
+        <v>478</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G2" s="7"/>
+      <c r="G2" s="8"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>480</v>
+      <c r="C3" s="10" t="s">
+        <v>481</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>482</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>484</v>
+      <c r="C4" s="10" t="s">
+        <v>486</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>118</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>20</v>
@@ -7108,62 +7162,62 @@
         <v>20</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>118</v>
@@ -7172,19 +7226,19 @@
     </row>
     <row r="24" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>118</v>
@@ -7193,306 +7247,306 @@
     </row>
     <row r="25" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>545</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>546</v>
+      <c r="C25" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>548</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>548</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>548</v>
+      <c r="C26" s="11" t="s">
+        <v>550</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>550</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>118</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>296</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>118</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>289</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>290</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>291</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>292</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>499</v>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>559</v>
+        <v>501</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>561</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>293</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>294</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>564</v>
+        <v>484</v>
+      </c>
+      <c r="H33" s="13" t="s">
+        <v>566</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>295</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>298</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>573</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>28</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="5"/>
+      <c r="B37" s="6"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="5"/>
+      <c r="B38" s="6"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="5"/>
+      <c r="B39" s="6"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -7523,7 +7577,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -7541,7 +7595,7 @@
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7758,7 +7812,7 @@
         <v>100</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>33</v>
@@ -7778,7 +7832,7 @@
         <v>101</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>33</v>
@@ -7798,7 +7852,7 @@
         <v>102</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>33</v>
@@ -7818,7 +7872,7 @@
         <v>103</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>33</v>
@@ -7838,7 +7892,7 @@
         <v>104</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>33</v>
@@ -7858,7 +7912,7 @@
         <v>105</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>33</v>
@@ -7872,13 +7926,13 @@
         <v>104</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>106</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>33</v>
@@ -7898,13 +7952,13 @@
         <v>107</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7921,13 +7975,13 @@
         <v>108</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7944,7 +7998,7 @@
         <v>109</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>33</v>
@@ -7964,13 +8018,13 @@
         <v>107</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7987,7 +8041,7 @@
         <v>110</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>33</v>
@@ -8007,7 +8061,7 @@
         <v>111</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>34</v>
@@ -8027,13 +8081,13 @@
         <v>107</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8050,7 +8104,7 @@
         <v>108</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>33</v>
@@ -8070,7 +8124,7 @@
         <v>112</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>33</v>
@@ -8090,7 +8144,7 @@
         <v>113</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>33</v>
@@ -8110,7 +8164,7 @@
         <v>114</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>118</v>
@@ -8130,7 +8184,7 @@
         <v>115</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>33</v>
@@ -8150,7 +8204,7 @@
         <v>116</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>33</v>
@@ -8170,7 +8224,7 @@
         <v>117</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>33</v>
@@ -8190,7 +8244,7 @@
         <v>107</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>33</v>
@@ -8210,7 +8264,7 @@
         <v>118</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>33</v>
@@ -8230,7 +8284,7 @@
         <v>119</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>34</v>
@@ -8250,7 +8304,7 @@
         <v>120</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>33</v>
@@ -8270,7 +8324,7 @@
         <v>129</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>33</v>
@@ -8290,7 +8344,7 @@
         <v>128</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>33</v>
@@ -8310,7 +8364,7 @@
         <v>121</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>33</v>
@@ -8330,7 +8384,7 @@
         <v>122</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>33</v>
@@ -8350,7 +8404,7 @@
         <v>121</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>33</v>
@@ -8370,7 +8424,7 @@
         <v>123</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>33</v>
@@ -8390,7 +8444,7 @@
         <v>124</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>33</v>
@@ -8410,13 +8464,13 @@
         <v>125</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8433,7 +8487,7 @@
         <v>6</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>330</v>
+        <v>583</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>33</v>
@@ -8453,7 +8507,7 @@
         <v>126</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>33</v>
@@ -8473,7 +8527,7 @@
         <v>127</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>33</v>
@@ -8533,7 +8587,7 @@
         <v>7</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>33</v>
@@ -8566,25 +8620,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8598,16 +8652,16 @@
         <v>25</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="I2" s="1"/>
     </row>
@@ -8622,16 +8676,16 @@
         <v>25</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="I3" s="1"/>
     </row>
@@ -8646,16 +8700,16 @@
         <v>160</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="I4" s="1"/>
     </row>
@@ -8670,13 +8724,13 @@
         <v>160</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="I5" s="1"/>
     </row>
@@ -8691,13 +8745,13 @@
         <v>224</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="I6" s="1"/>
     </row>
@@ -8709,19 +8763,19 @@
         <v>246</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>160</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="I7" s="1"/>
     </row>
@@ -8736,13 +8790,13 @@
         <v>160</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -8776,25 +8830,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>571</v>
+        <v>506</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>573</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8802,39 +8856,39 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>617</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>618</v>
+        <v>620</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>621</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>620</v>
+      <c r="B3" s="6" t="s">
+        <v>623</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8842,19 +8896,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8862,19 +8916,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>627</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>618</v>
+        <v>630</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>621</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8882,19 +8936,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8902,19 +8956,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>634</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>631</v>
-      </c>
       <c r="F7" s="1" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8922,19 +8976,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>618</v>
+        <v>640</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>621</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8942,19 +8996,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8962,19 +9016,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8982,19 +9036,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9002,19 +9056,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9022,19 +9076,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9042,22 +9096,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9065,22 +9119,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9088,19 +9142,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>663</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>618</v>
+        <v>666</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>621</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9108,19 +9162,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>279</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
     </row>
   </sheetData>
@@ -9149,145 +9203,145 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>672</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>203</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9367,13 +9421,13 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="F1" s="1"/>
-      <c r="G1" s="5"/>
+      <c r="G1" s="6"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9387,7 +9441,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="F2" s="1"/>
       <c r="H2" s="1"/>
@@ -9403,7 +9457,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="F3" s="1"/>
       <c r="H3" s="1"/>
@@ -9419,7 +9473,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" s="1"/>
@@ -9435,7 +9489,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>
@@ -9451,7 +9505,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="1"/>
@@ -9467,7 +9521,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="1"/>
@@ -9483,7 +9537,7 @@
         <v>3</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1"/>
@@ -9499,7 +9553,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="F9" s="1"/>
       <c r="H9" s="1"/>
@@ -9515,7 +9569,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1"/>
@@ -9531,7 +9585,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1"/>
@@ -9547,10 +9601,10 @@
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="F12" s="1"/>
-      <c r="G12" s="5"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9564,10 +9618,10 @@
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="F13" s="1"/>
-      <c r="G13" s="5"/>
+      <c r="G13" s="6"/>
       <c r="H13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9581,10 +9635,10 @@
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="F14" s="1"/>
-      <c r="G14" s="5"/>
+      <c r="G14" s="6"/>
       <c r="H14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9598,7 +9652,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="F15" s="1"/>
       <c r="H15" s="1"/>
@@ -9608,13 +9662,13 @@
         <v>104</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1"/>
@@ -9630,7 +9684,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1"/>
@@ -9646,7 +9700,7 @@
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="F18" s="1"/>
       <c r="H18" s="1"/>
@@ -9662,7 +9716,7 @@
         <v>9</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9676,7 +9730,7 @@
         <v>8</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -9692,7 +9746,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9706,7 +9760,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9720,7 +9774,7 @@
         <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9734,7 +9788,7 @@
         <v>8</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9748,7 +9802,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9762,7 +9816,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9776,7 +9830,7 @@
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9790,7 +9844,7 @@
         <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9804,7 +9858,7 @@
         <v>12</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9818,7 +9872,7 @@
         <v>12</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9832,7 +9886,7 @@
         <v>15</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9846,7 +9900,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9860,7 +9914,7 @@
         <v>13</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9874,7 +9928,7 @@
         <v>14</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9888,7 +9942,7 @@
         <v>14</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9902,7 +9956,7 @@
         <v>13</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9916,7 +9970,7 @@
         <v>13</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9930,7 +9984,7 @@
         <v>16</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update : ajout point de vigilance BBR , capacité de production et ADOPE
</commit_message>
<xml_diff>
--- a/fiches indicateurs.xlsx
+++ b/fiches indicateurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="indicateurs" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="706">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1868" uniqueCount="709">
   <si>
     <t xml:space="preserve">fiche_indicateur</t>
   </si>
@@ -2201,6 +2201,15 @@
   </si>
   <si>
     <t xml:space="preserve">Risque de données non homogènes si l'on croise la "Surface érosion" de l'OEIL avec le "Terrain nu" issu du MOS ,  le MOS est privilégié pour sa robustesse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, 500, 503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le BBR intègre le volume de prélèvement autorisé et le débits caractéristiques d’étiage médian (DCE2).</t>
   </si>
   <si>
     <t xml:space="preserve">Sous-groupe d'objectif</t>
@@ -5518,7 +5527,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
@@ -9344,6 +9353,20 @@
         <v>700</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>703</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -9424,7 +9447,7 @@
         <v>615</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="6"/>
@@ -9569,7 +9592,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1"/>
@@ -9585,7 +9608,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1"/>
@@ -9716,7 +9739,7 @@
         <v>9</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9858,7 +9881,7 @@
         <v>12</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9872,7 +9895,7 @@
         <v>12</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9984,7 +10007,7 @@
         <v>16</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix adaptation glossaire couverture spatiale
</commit_message>
<xml_diff>
--- a/fiches indicateurs.xlsx
+++ b/fiches indicateurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="indicateurs" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1868" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="710">
   <si>
     <t xml:space="preserve">fiche_indicateur</t>
   </si>
@@ -1028,34 +1028,7 @@
     <t xml:space="preserve">https://www.arcgis.com/home/item.html?id=6d48f295daf5471a842054d9e050765d</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">La couche BBR (bilan besoin / ressources) est calculée à partir des débits caractéristiques d’étiage médian (DCE2) auquel sont soustraits l'ensemble des </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">prélèvements d’eau autorisés</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
+    <t xml:space="preserve">La couche BBR (bilan besoin / ressources) est calculée à partir des débits caractéristiques d’étiage médian (DCE2) auquel sont soustraits l'ensemble des prélèvements d’eau autorisés.</t>
   </si>
   <si>
     <t xml:space="preserve">https://georep.nc/actualites/nouvelle-donnee-en-hydrologie-le-bilan-besoin-ressource</t>
@@ -1788,7 +1761,10 @@
     <t xml:space="preserve">Couverture spatiale</t>
   </si>
   <si>
-    <t xml:space="preserve">Couverture spatiale de la donnée</t>
+    <t xml:space="preserve">Désigne l'étendue géographique ou l'emprise territoriale sur laquelle la donnée source est disponible et valide. Cet attribut permet à l'utilisateur de savoir si l'indicateur est calculé sur l'ensemble de la Nouvelle-Calédonie, sur une province spécifique (ex: Province Sud) ou uniquement sur un périmètre restreint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nouvelle-Calédonie / provinces / communes … </t>
   </si>
   <si>
     <t xml:space="preserve">Période d actualisation</t>
@@ -2332,7 +2308,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2353,7 +2329,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2383,6 +2359,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -5527,7 +5507,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
@@ -6641,7 +6621,7 @@
   </sheetData>
   <autoFilter ref="A1:L38"/>
   <hyperlinks>
-    <hyperlink ref="J7" r:id="rId1" display="prélèvements d’eau autorisés"/>
+    <hyperlink ref="J7" r:id="rId1" display="La couche BBR (bilan besoin / ressources) est calculée à partir des débits caractéristiques d’étiage médian (DCE2) auquel sont soustraits l'ensemble des prélèvements d’eau autorisés."/>
     <hyperlink ref="E33" r:id="rId2" display="https://georep-dtsi-sgt.opendata.arcgis.com/documents/d7ab36bb69954aea882a63993428357a/about"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -7431,7 +7411,7 @@
       <c r="C32" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" s="13" t="s">
         <v>563</v>
       </c>
       <c r="E32" s="1" t="s">
@@ -7442,6 +7422,9 @@
       </c>
       <c r="G32" s="3" t="s">
         <v>501</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>564</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7452,10 +7435,10 @@
         <v>294</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>552</v>
@@ -7466,8 +7449,8 @@
       <c r="G33" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="H33" s="13" t="s">
-        <v>566</v>
+      <c r="H33" s="14" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7478,10 +7461,10 @@
         <v>295</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>519</v>
@@ -7493,7 +7476,7 @@
         <v>484</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7504,10 +7487,10 @@
         <v>298</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>500</v>
@@ -7521,16 +7504,16 @@
     </row>
     <row r="36" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>500</v>
@@ -7586,7 +7569,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -7604,7 +7587,7 @@
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7935,7 +7918,7 @@
         <v>104</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>106</v>
@@ -7967,7 +7950,7 @@
         <v>33</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7990,7 +7973,7 @@
         <v>33</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8033,7 +8016,7 @@
         <v>33</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8096,7 +8079,7 @@
         <v>33</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8479,7 +8462,7 @@
         <v>34</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8496,7 +8479,7 @@
         <v>6</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>33</v>
@@ -8596,7 +8579,7 @@
         <v>7</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>33</v>
@@ -8629,25 +8612,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>489</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8661,16 +8644,16 @@
         <v>25</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="I2" s="1"/>
     </row>
@@ -8685,16 +8668,16 @@
         <v>25</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="I3" s="1"/>
     </row>
@@ -8709,16 +8692,16 @@
         <v>160</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="I4" s="1"/>
     </row>
@@ -8733,13 +8716,13 @@
         <v>160</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="I5" s="1"/>
     </row>
@@ -8754,13 +8737,13 @@
         <v>224</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I6" s="1"/>
     </row>
@@ -8772,19 +8755,19 @@
         <v>246</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>160</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="I7" s="1"/>
     </row>
@@ -8799,13 +8782,13 @@
         <v>160</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -8839,25 +8822,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>506</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8865,19 +8848,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8885,19 +8868,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8905,19 +8888,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8925,19 +8908,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8945,19 +8928,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8965,19 +8948,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8985,19 +8968,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9005,19 +8988,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9025,19 +9008,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9045,19 +9028,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9065,19 +9048,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9085,19 +9068,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9105,22 +9088,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9128,22 +9111,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9151,19 +9134,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9171,19 +9154,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>279</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
     </row>
   </sheetData>
@@ -9212,13 +9195,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>472</v>
@@ -9226,145 +9209,145 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>203</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>675</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>703</v>
+        <v>676</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9444,10 +9427,10 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="6"/>
@@ -9464,7 +9447,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F2" s="1"/>
       <c r="H2" s="1"/>
@@ -9480,7 +9463,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F3" s="1"/>
       <c r="H3" s="1"/>
@@ -9496,7 +9479,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" s="1"/>
@@ -9512,7 +9495,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>
@@ -9528,7 +9511,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="1"/>
@@ -9544,7 +9527,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="1"/>
@@ -9560,7 +9543,7 @@
         <v>3</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1"/>
@@ -9576,7 +9559,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="F9" s="1"/>
       <c r="H9" s="1"/>
@@ -9592,7 +9575,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1"/>
@@ -9608,7 +9591,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1"/>
@@ -9624,7 +9607,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="6"/>
@@ -9641,7 +9624,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="6"/>
@@ -9658,7 +9641,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="6"/>
@@ -9675,7 +9658,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="F15" s="1"/>
       <c r="H15" s="1"/>
@@ -9685,13 +9668,13 @@
         <v>104</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1"/>
@@ -9707,7 +9690,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1"/>
@@ -9723,7 +9706,7 @@
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F18" s="1"/>
       <c r="H18" s="1"/>
@@ -9739,7 +9722,7 @@
         <v>9</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9753,7 +9736,7 @@
         <v>8</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -9769,7 +9752,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9783,7 +9766,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9797,7 +9780,7 @@
         <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9811,7 +9794,7 @@
         <v>8</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9825,7 +9808,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9839,7 +9822,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9853,7 +9836,7 @@
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9867,7 +9850,7 @@
         <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9881,7 +9864,7 @@
         <v>12</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9895,7 +9878,7 @@
         <v>12</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9909,7 +9892,7 @@
         <v>15</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9923,7 +9906,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9937,7 +9920,7 @@
         <v>13</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9951,7 +9934,7 @@
         <v>14</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9965,7 +9948,7 @@
         <v>14</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9979,7 +9962,7 @@
         <v>13</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9993,7 +9976,7 @@
         <v>13</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10007,7 +9990,7 @@
         <v>16</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix : modification des nom des indicateur AODPE
</commit_message>
<xml_diff>
--- a/fiches indicateurs.xlsx
+++ b/fiches indicateurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="indicateurs" sheetId="1" state="visible" r:id="rId3"/>
@@ -16,6 +16,7 @@
     <sheet name="groupes" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="vigilances" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="relation groupe objectifs" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Famille" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">sources!$A$1:$L$38</definedName>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1882" uniqueCount="719">
   <si>
     <t xml:space="preserve">fiche_indicateur</t>
   </si>
@@ -833,7 +834,7 @@
     <t xml:space="preserve">Niveau bas = forte criticité quantitative</t>
   </si>
   <si>
-    <t xml:space="preserve">AODPE nombre</t>
+    <t xml:space="preserve">Nombre de prélèvement AODPE</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre de prélèvements d’eau autorisés.</t>
@@ -851,7 +852,23 @@
     <t xml:space="preserve">Indicateur pression captage. Donnée dynamique DAVAR. Intégrable en analyse.</t>
   </si>
   <si>
-    <t xml:space="preserve">AODPE volume</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Volume des p</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">rélèvements AODPE</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Volume total d’eau prélevé.</t>
@@ -1828,6 +1845,12 @@
     <t xml:space="preserve">Bilan Besoin Ressource (nom à vérifier)</t>
   </si>
   <si>
+    <t xml:space="preserve">AODPE nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AODPE volume</t>
+  </si>
+  <si>
     <t xml:space="preserve">Base de données ATYA (nom à vérifier)</t>
   </si>
   <si>
@@ -2201,6 +2224,27 @@
   </si>
   <si>
     <t xml:space="preserve">État sanitaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cette famille regroupe les indicateurs qui caractérisent la valeur stratégique et la résilience des systèmes d’eau potable. Ils servent de « contrepoids » aux menaces pour déterminer la criticité globale d'un captage en quantifiant ce qui doit être protégé (population, infrastructures, biodiversité dépendante)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qu'est-ce qu'on protège ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cette famille identifie les menaces actives et les aléas, d’origine humaine ou naturelle, susceptibles d’affaiblir les ressources. Elle mesure l'intensité des agressions (incendies, urbanisation, prélèvements) que subit le bassin versant et qui peuvent rompre les processus naturels de régulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qu'est-ce qui menace ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cette famille définit le socle physique immuable et les caractéristiques internes des captages qui expliquent leur sensibilité intrinsèque. Contrairement aux pressions, elle ne mesure pas un événement mais la prédisposition naturelle du terrain (géologie, type d'ouvrage) à laisser circuler ou non des polluants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">à quel point le système est sensible ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contexte / État</t>
   </si>
 </sst>
 </file>
@@ -2210,7 +2254,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2237,6 +2281,11 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2308,7 +2357,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2330,7 +2379,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -2338,10 +2387,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2357,7 +2410,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2365,8 +2418,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -5139,7 +5196,7 @@
       <c r="D38" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="5" t="s">
         <v>273</v>
       </c>
       <c r="F38" s="1" t="s">
@@ -5535,7 +5592,7 @@
       <c r="I7" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="6" t="s">
         <v>332</v>
       </c>
       <c r="K7" s="1" t="s">
@@ -6115,7 +6172,7 @@
       <c r="G24" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="7" t="s">
         <v>412</v>
       </c>
       <c r="I24" s="1" t="s">
@@ -6418,7 +6475,7 @@
       <c r="D33" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="8" t="s">
         <v>442</v>
       </c>
       <c r="F33" s="1" t="s">
@@ -6658,7 +6715,7 @@
       <c r="B1" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>471</v>
       </c>
       <c r="D1" s="3" t="s">
@@ -6670,7 +6727,7 @@
       <c r="F1" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="9" t="s">
         <v>475</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -6684,7 +6741,7 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="10" t="s">
         <v>478</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -6696,7 +6753,7 @@
       <c r="F2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G2" s="8"/>
+      <c r="G2" s="9"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6706,10 +6763,10 @@
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="11" t="s">
         <v>481</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="11" t="s">
         <v>482</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -6732,7 +6789,7 @@
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>486</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -7241,10 +7298,10 @@
       <c r="B25" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>547</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="11" t="s">
         <v>548</v>
       </c>
       <c r="E25" s="1" t="s">
@@ -7267,10 +7324,10 @@
       <c r="B26" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="12" t="s">
         <v>550</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="12" t="s">
         <v>550</v>
       </c>
       <c r="E26" s="1" t="s">
@@ -7397,7 +7454,7 @@
       <c r="G31" s="3" t="s">
         <v>501</v>
       </c>
-      <c r="H31" s="12" t="s">
+      <c r="H31" s="13" t="s">
         <v>561</v>
       </c>
     </row>
@@ -7411,7 +7468,7 @@
       <c r="C32" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="14" t="s">
         <v>563</v>
       </c>
       <c r="E32" s="1" t="s">
@@ -7449,7 +7506,7 @@
       <c r="G33" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="H33" s="14" t="s">
+      <c r="H33" s="15" t="s">
         <v>567</v>
       </c>
     </row>
@@ -7506,7 +7563,7 @@
       <c r="A36" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>574</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -7526,19 +7583,19 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6"/>
+      <c r="B37" s="7"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="6"/>
+      <c r="B38" s="7"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="14.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="6"/>
+      <c r="B39" s="7"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -8533,7 +8590,7 @@
         <v>503</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>267</v>
+        <v>585</v>
       </c>
       <c r="D48" s="1" t="n">
         <v>3</v>
@@ -8553,7 +8610,7 @@
         <v>504</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>273</v>
+        <v>586</v>
       </c>
       <c r="D49" s="1" t="n">
         <v>3</v>
@@ -8579,7 +8636,7 @@
         <v>7</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>33</v>
@@ -8612,25 +8669,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>489</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8644,16 +8701,16 @@
         <v>25</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="I2" s="1"/>
     </row>
@@ -8668,16 +8725,16 @@
         <v>25</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="I3" s="1"/>
     </row>
@@ -8692,16 +8749,16 @@
         <v>160</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="I4" s="1"/>
     </row>
@@ -8716,13 +8773,13 @@
         <v>160</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I5" s="1"/>
     </row>
@@ -8737,13 +8794,13 @@
         <v>224</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="I6" s="1"/>
     </row>
@@ -8755,19 +8812,19 @@
         <v>246</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>160</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="I7" s="1"/>
     </row>
@@ -8782,13 +8839,13 @@
         <v>160</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -8822,25 +8879,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>573</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>574</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8848,39 +8905,39 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>621</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>622</v>
+        <v>623</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>624</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>624</v>
+      <c r="B3" s="7" t="s">
+        <v>626</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8888,19 +8945,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8908,19 +8965,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>631</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>622</v>
+        <v>633</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>624</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8928,19 +8985,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8948,19 +9005,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8968,19 +9025,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>641</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>622</v>
+        <v>643</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>624</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8988,19 +9045,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9008,19 +9065,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>159</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9028,19 +9085,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9048,19 +9105,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9068,19 +9125,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>188</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9088,22 +9145,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9111,22 +9168,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>246</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9134,19 +9191,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>667</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>622</v>
+        <v>669</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>624</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9154,19 +9211,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>279</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>500</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
   </sheetData>
@@ -9198,10 +9255,10 @@
         <v>577</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>472</v>
@@ -9209,145 +9266,145 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>678</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>679</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>676</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>203</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9427,13 +9484,13 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="F1" s="1"/>
-      <c r="G1" s="6"/>
+      <c r="G1" s="7"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9447,7 +9504,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="F2" s="1"/>
       <c r="H2" s="1"/>
@@ -9463,7 +9520,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="F3" s="1"/>
       <c r="H3" s="1"/>
@@ -9479,7 +9536,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" s="1"/>
@@ -9495,7 +9552,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>
@@ -9511,7 +9568,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" s="1"/>
@@ -9527,7 +9584,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="1"/>
@@ -9543,7 +9600,7 @@
         <v>3</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1"/>
@@ -9559,7 +9616,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F9" s="1"/>
       <c r="H9" s="1"/>
@@ -9575,7 +9632,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1"/>
@@ -9591,7 +9648,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1"/>
@@ -9607,10 +9664,10 @@
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F12" s="1"/>
-      <c r="G12" s="6"/>
+      <c r="G12" s="7"/>
       <c r="H12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9624,10 +9681,10 @@
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F13" s="1"/>
-      <c r="G13" s="6"/>
+      <c r="G13" s="7"/>
       <c r="H13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9641,10 +9698,10 @@
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="F14" s="1"/>
-      <c r="G14" s="6"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9658,7 +9715,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="F15" s="1"/>
       <c r="H15" s="1"/>
@@ -9674,7 +9731,7 @@
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1"/>
@@ -9690,7 +9747,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1"/>
@@ -9706,7 +9763,7 @@
         <v>7</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="F18" s="1"/>
       <c r="H18" s="1"/>
@@ -9722,7 +9779,7 @@
         <v>9</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9736,7 +9793,7 @@
         <v>8</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -9752,7 +9809,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9766,7 +9823,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9780,7 +9837,7 @@
         <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9794,7 +9851,7 @@
         <v>8</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9808,7 +9865,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9822,7 +9879,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9836,7 +9893,7 @@
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9850,7 +9907,7 @@
         <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9864,7 +9921,7 @@
         <v>12</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9878,7 +9935,7 @@
         <v>12</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9892,7 +9949,7 @@
         <v>15</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9906,7 +9963,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9920,7 +9977,7 @@
         <v>13</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9934,7 +9991,7 @@
         <v>14</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9948,7 +10005,7 @@
         <v>14</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9956,13 +10013,13 @@
         <v>503</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>267</v>
+        <v>585</v>
       </c>
       <c r="C36" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9970,13 +10027,13 @@
         <v>504</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>273</v>
+        <v>586</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9990,7 +10047,79 @@
         <v>16</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>709</v>
+        <v>711</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.89"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>712</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>714</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="75.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>716</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>